<commit_message>
Aggiungi file FIGLIO con le 24 sedute esplose + rimando dal PADRE
Struttura padre-figlio:
- PADRE (Programma_PreSeason_VolleyD.xlsx): strategia/manuale (aggiunto
  rimando al figlio).
- FIGLIO (Sedute_PreSeason_VolleyD.xlsx): operativo. Indice + 8 fogli
  settimana (S1-S8) con le 3 sedute esplose esercizio per esercizio
  (tempi, S×R, RPE, kg/%1RM, varianti Rosso/Verde), colonna 'Note &
  modifiche per atleta' in ogni riga + foglio 'Registro modifiche'
  strutturato. Nessun roster (come richiesto).
- build_sedute.py (generatore).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013QVzQE1AzZA84pgyx3jja2
</commit_message>
<xml_diff>
--- a/programmi/preseason_volley_serieD/Programma_PreSeason_VolleyD.xlsx
+++ b/programmi/preseason_volley_serieD/Programma_PreSeason_VolleyD.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,6 +68,10 @@
     </font>
     <font>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F7A1F"/>
     </font>
   </fonts>
   <fills count="9">
@@ -183,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -283,6 +287,7 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -677,6 +682,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="B3" s="35" t="inlineStr">
+        <is>
+          <t>▶ File collegato (FIGLIO · sedute operative esplose): 'Sedute_PreSeason_VolleyD.xlsx'</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
@@ -695,6 +707,13 @@
           <t>Serie D femminile · atlete 18–32 anni</t>
         </is>
       </c>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="24" t="n"/>
+      <c r="G5" s="24" t="n"/>
+      <c r="H5" s="24" t="n"/>
+      <c r="I5" s="24" t="n"/>
+      <c r="J5" s="25" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
@@ -707,6 +726,13 @@
           <t>Eterogenei: forma variabile; alcune equilibrate, altre con problemi motori → 3 fasce (Rosso/Giallo/Verde)</t>
         </is>
       </c>
+      <c r="D6" s="24" t="n"/>
+      <c r="E6" s="24" t="n"/>
+      <c r="F6" s="24" t="n"/>
+      <c r="G6" s="24" t="n"/>
+      <c r="H6" s="24" t="n"/>
+      <c r="I6" s="24" t="n"/>
+      <c r="J6" s="25" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
@@ -719,6 +745,13 @@
           <t>3 sedute/settimana · 2 Campo + 1 Pesi · durata media 60'</t>
         </is>
       </c>
+      <c r="D7" s="24" t="n"/>
+      <c r="E7" s="24" t="n"/>
+      <c r="F7" s="24" t="n"/>
+      <c r="G7" s="24" t="n"/>
+      <c r="H7" s="24" t="n"/>
+      <c r="I7" s="24" t="n"/>
+      <c r="J7" s="25" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="4" t="inlineStr">
@@ -731,6 +764,13 @@
           <t>Elastici, skimmy (mini-band), TRX, ostacoli, coni/cinesini, box</t>
         </is>
       </c>
+      <c r="D8" s="24" t="n"/>
+      <c r="E8" s="24" t="n"/>
+      <c r="F8" s="24" t="n"/>
+      <c r="G8" s="24" t="n"/>
+      <c r="H8" s="24" t="n"/>
+      <c r="I8" s="24" t="n"/>
+      <c r="J8" s="25" t="n"/>
     </row>
     <row r="9">
       <c r="B9" s="4" t="inlineStr">
@@ -743,6 +783,13 @@
           <t>Palestra completa</t>
         </is>
       </c>
+      <c r="D9" s="24" t="n"/>
+      <c r="E9" s="24" t="n"/>
+      <c r="F9" s="24" t="n"/>
+      <c r="G9" s="24" t="n"/>
+      <c r="H9" s="24" t="n"/>
+      <c r="I9" s="24" t="n"/>
+      <c r="J9" s="25" t="n"/>
     </row>
     <row r="10">
       <c r="B10" s="4" t="inlineStr">
@@ -755,6 +802,13 @@
           <t>Sviluppare la condizione con progressioni proporzionali e crescenti; forza + potenza sport-specifica + prevenzione</t>
         </is>
       </c>
+      <c r="D10" s="24" t="n"/>
+      <c r="E10" s="24" t="n"/>
+      <c r="F10" s="24" t="n"/>
+      <c r="G10" s="24" t="n"/>
+      <c r="H10" s="24" t="n"/>
+      <c r="I10" s="24" t="n"/>
+      <c r="J10" s="25" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="4" t="inlineStr">
@@ -767,6 +821,13 @@
           <t>Preparazione 01/09 → 25/10 · 1ª gara sab 31/10</t>
         </is>
       </c>
+      <c r="D11" s="24" t="n"/>
+      <c r="E11" s="24" t="n"/>
+      <c r="F11" s="24" t="n"/>
+      <c r="G11" s="24" t="n"/>
+      <c r="H11" s="24" t="n"/>
+      <c r="I11" s="24" t="n"/>
+      <c r="J11" s="25" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
@@ -1176,6 +1237,12 @@
           <t>Riscaldamento neuromuscolare · agilità/pliometria · condizionamento · prevenzione</t>
         </is>
       </c>
+      <c r="E29" s="24" t="n"/>
+      <c r="F29" s="24" t="n"/>
+      <c r="G29" s="24" t="n"/>
+      <c r="H29" s="24" t="n"/>
+      <c r="I29" s="24" t="n"/>
+      <c r="J29" s="25" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="4" t="inlineStr">
@@ -1193,6 +1260,12 @@
           <t>—</t>
         </is>
       </c>
+      <c r="E30" s="24" t="n"/>
+      <c r="F30" s="24" t="n"/>
+      <c r="G30" s="24" t="n"/>
+      <c r="H30" s="24" t="n"/>
+      <c r="I30" s="24" t="n"/>
+      <c r="J30" s="25" t="n"/>
     </row>
     <row r="31">
       <c r="B31" s="4" t="inlineStr">
@@ -1210,6 +1283,12 @@
           <t>Fondamentali (squat/hinge/spinta/tirata) · core · prevenzione</t>
         </is>
       </c>
+      <c r="E31" s="24" t="n"/>
+      <c r="F31" s="24" t="n"/>
+      <c r="G31" s="24" t="n"/>
+      <c r="H31" s="24" t="n"/>
+      <c r="I31" s="24" t="n"/>
+      <c r="J31" s="25" t="n"/>
     </row>
     <row r="32">
       <c r="B32" s="4" t="inlineStr">
@@ -1227,6 +1306,12 @@
           <t>—</t>
         </is>
       </c>
+      <c r="E32" s="24" t="n"/>
+      <c r="F32" s="24" t="n"/>
+      <c r="G32" s="24" t="n"/>
+      <c r="H32" s="24" t="n"/>
+      <c r="I32" s="24" t="n"/>
+      <c r="J32" s="25" t="n"/>
     </row>
     <row r="33">
       <c r="B33" s="4" t="inlineStr">
@@ -1244,6 +1329,12 @@
           <t>Riscaldamento neuromusc. · blocco forza (unilaterale/post./prev.) · gesto specifico · condizionamento specifico</t>
         </is>
       </c>
+      <c r="E33" s="24" t="n"/>
+      <c r="F33" s="24" t="n"/>
+      <c r="G33" s="24" t="n"/>
+      <c r="H33" s="24" t="n"/>
+      <c r="I33" s="24" t="n"/>
+      <c r="J33" s="25" t="n"/>
     </row>
     <row r="34">
       <c r="B34" s="4" t="inlineStr">
@@ -1261,6 +1352,12 @@
           <t>In fase gara: sab 31/10 1ª partita</t>
         </is>
       </c>
+      <c r="E34" s="24" t="n"/>
+      <c r="F34" s="24" t="n"/>
+      <c r="G34" s="24" t="n"/>
+      <c r="H34" s="24" t="n"/>
+      <c r="I34" s="24" t="n"/>
+      <c r="J34" s="25" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -1324,6 +1421,9 @@
           <t>Sforzo percepito 0–10 (10 = massimo, nessuna ripetizione di riserva). Guida principale del carico.</t>
         </is>
       </c>
+      <c r="D4" s="24" t="n"/>
+      <c r="E4" s="24" t="n"/>
+      <c r="F4" s="25" t="n"/>
     </row>
     <row r="5">
       <c r="B5" s="4" t="inlineStr">
@@ -1336,6 +1436,9 @@
           <t>Percentuale del massimale (per gli esercizi di sala). I kg sono calcolati su un 1RM di RIFERIMENTO.</t>
         </is>
       </c>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="25" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
@@ -1348,6 +1451,9 @@
           <t>Serie × Ripetizioni</t>
         </is>
       </c>
+      <c r="D6" s="24" t="n"/>
+      <c r="E6" s="24" t="n"/>
+      <c r="F6" s="25" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
@@ -1360,6 +1466,9 @@
           <t>Recupero tra le serie</t>
         </is>
       </c>
+      <c r="D7" s="24" t="n"/>
+      <c r="E7" s="24" t="n"/>
+      <c r="F7" s="25" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="4" t="inlineStr">
@@ -1372,6 +1481,9 @@
           <t>🔴 Rosso = regressioni (decondizionate/problemi motori) · 🟡 Giallo = base · 🟢 Verde = progressioni</t>
         </is>
       </c>
+      <c r="D8" s="24" t="n"/>
+      <c r="E8" s="24" t="n"/>
+      <c r="F8" s="25" t="n"/>
     </row>
     <row r="9">
       <c r="B9" s="4" t="inlineStr">
@@ -1384,6 +1496,9 @@
           <t>Protocollo fisso tipo FIFA 11+ adattato: attivazione, controllo atterraggio, core (5–8')</t>
         </is>
       </c>
+      <c r="D9" s="24" t="n"/>
+      <c r="E9" s="24" t="n"/>
+      <c r="F9" s="25" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="3" t="inlineStr">
@@ -1505,6 +1620,9 @@
           <t>Corpo libero/manubri leggeri, ROM controllato, atterraggi (non salti), supporti (TRX/box), volumi ridotti, RPE 5–6. Sale quando il movimento è pulito.</t>
         </is>
       </c>
+      <c r="D19" s="24" t="n"/>
+      <c r="E19" s="24" t="n"/>
+      <c r="F19" s="25" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="4" t="inlineStr">
@@ -1517,6 +1635,9 @@
           <t>Versione standard, RPE 6–8. Riferimento del programma.</t>
         </is>
       </c>
+      <c r="D20" s="24" t="n"/>
+      <c r="E20" s="24" t="n"/>
+      <c r="F20" s="25" t="n"/>
     </row>
     <row r="21">
       <c r="B21" s="4" t="inlineStr">
@@ -1529,6 +1650,9 @@
           <t>Carico/bilanciere, salti e ri-salti, cluster, velocità, %1RM, RPE 7–9 (mai cedimento in preparazione).</t>
         </is>
       </c>
+      <c r="D21" s="24" t="n"/>
+      <c r="E21" s="24" t="n"/>
+      <c r="F21" s="25" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -1592,6 +1716,11 @@
           <t>Valutare e mettere in sicurezza (screening, atterraggi, mobilità), costruire capacità di lavoro e forza generale; introdurre agilità e salti bassi. Carichi bassi, qualità massima; volume crescente S1→S3.</t>
         </is>
       </c>
+      <c r="C5" s="24" t="n"/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="24" t="n"/>
+      <c r="G5" s="25" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
@@ -2363,6 +2492,11 @@
           <t>• Pliometria: S1 atterraggi/soft landing · S2 atterraggi + salti bassi 3×5 · S3 salti bassi + intro ostacolo. Gate per salire: atterraggio allineato e indolore.</t>
         </is>
       </c>
+      <c r="C40" s="24" t="n"/>
+      <c r="D40" s="24" t="n"/>
+      <c r="E40" s="24" t="n"/>
+      <c r="F40" s="24" t="n"/>
+      <c r="G40" s="25" t="n"/>
     </row>
     <row r="41">
       <c r="B41" s="5" t="inlineStr">
@@ -2370,6 +2504,11 @@
           <t>• Condizionamento generale: navette 6→8; circuiti 3 giri. RPE 6→7.</t>
         </is>
       </c>
+      <c r="C41" s="24" t="n"/>
+      <c r="D41" s="24" t="n"/>
+      <c r="E41" s="24" t="n"/>
+      <c r="F41" s="24" t="n"/>
+      <c r="G41" s="25" t="n"/>
     </row>
     <row r="42">
       <c r="B42" s="5" t="inlineStr">
@@ -2377,6 +2516,11 @@
           <t>• Forza campo (Campo B): volume 2→3-4 serie su unilaterale/catena post./Nordic. È il 2° stimolo forza settimanale.</t>
         </is>
       </c>
+      <c r="C42" s="24" t="n"/>
+      <c r="D42" s="24" t="n"/>
+      <c r="E42" s="24" t="n"/>
+      <c r="F42" s="24" t="n"/>
+      <c r="G42" s="25" t="n"/>
     </row>
     <row r="43">
       <c r="B43" s="5" t="inlineStr">
@@ -2384,6 +2528,11 @@
           <t>• Prevenzione: volume in crescita; Nordic eccentrico progressione settimanale (focus LCA).</t>
         </is>
       </c>
+      <c r="C43" s="24" t="n"/>
+      <c r="D43" s="24" t="n"/>
+      <c r="E43" s="24" t="n"/>
+      <c r="F43" s="24" t="n"/>
+      <c r="G43" s="25" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -2445,6 +2594,11 @@
           <t>Scarico programmato (riposo pulsato): −40% volume, intensità mantenuta ma senza cedimento. Recupero, consolidamento tecnico e RE-CHECK delle fasce prima del blocco intenso.</t>
         </is>
       </c>
+      <c r="C5" s="24" t="n"/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="24" t="n"/>
+      <c r="G5" s="25" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
@@ -3088,6 +3242,11 @@
           <t>• Pliometria: solo atterraggi di qualità. Nessun salto massimale.</t>
         </is>
       </c>
+      <c r="C38" s="24" t="n"/>
+      <c r="D38" s="24" t="n"/>
+      <c r="E38" s="24" t="n"/>
+      <c r="F38" s="24" t="n"/>
+      <c r="G38" s="25" t="n"/>
     </row>
     <row r="39">
       <c r="B39" s="5" t="inlineStr">
@@ -3095,6 +3254,11 @@
           <t>• Sala a volume ridotto (~65% / RPE6). Campo a 2 serie.</t>
         </is>
       </c>
+      <c r="C39" s="24" t="n"/>
+      <c r="D39" s="24" t="n"/>
+      <c r="E39" s="24" t="n"/>
+      <c r="F39" s="24" t="n"/>
+      <c r="G39" s="25" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="5" t="inlineStr">
@@ -3102,6 +3266,11 @@
           <t>• Obiettivo: arrivare fresche e riassegnare Rosso/Giallo/Verde per la Fase 2.</t>
         </is>
       </c>
+      <c r="C40" s="24" t="n"/>
+      <c r="D40" s="24" t="n"/>
+      <c r="E40" s="24" t="n"/>
+      <c r="F40" s="24" t="n"/>
+      <c r="G40" s="25" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -3162,6 +3331,11 @@
           <t>Sviluppo della forza (intensità ↑, reps ↓), pliometria estensiva strutturata → clusterizzata, condizionamento SPECIFICO volley, avvio trasferimento a potenza. Volume medio, intensità alta.</t>
         </is>
       </c>
+      <c r="C5" s="24" t="n"/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="24" t="n"/>
+      <c r="G5" s="25" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
@@ -3901,6 +4075,11 @@
           <t>• Pliometria: S5 estensiva strutturata · S6 clusterizzata (4+4+4, rec ampio) · S7 reattività + (🟢) intro intensiva leggera (drop basso) SOLO con gate forza (squat ~2×BW o profilo F-V).</t>
         </is>
       </c>
+      <c r="C39" s="24" t="n"/>
+      <c r="D39" s="24" t="n"/>
+      <c r="E39" s="24" t="n"/>
+      <c r="F39" s="24" t="n"/>
+      <c r="G39" s="25" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="5" t="inlineStr">
@@ -3908,6 +4087,11 @@
           <t>• Condizionamento SPECIFICO: salti/spostamenti ripetuti, simulazione attacco/muro, work:rest 1:2–1:3.</t>
         </is>
       </c>
+      <c r="C40" s="24" t="n"/>
+      <c r="D40" s="24" t="n"/>
+      <c r="E40" s="24" t="n"/>
+      <c r="F40" s="24" t="n"/>
+      <c r="G40" s="25" t="n"/>
     </row>
     <row r="41">
       <c r="B41" s="5" t="inlineStr">
@@ -3915,6 +4099,11 @@
           <t>• Forza campo: carico/tempo ↑ + salto caricato leggero (trasferimento).</t>
         </is>
       </c>
+      <c r="C41" s="24" t="n"/>
+      <c r="D41" s="24" t="n"/>
+      <c r="E41" s="24" t="n"/>
+      <c r="F41" s="24" t="n"/>
+      <c r="G41" s="25" t="n"/>
     </row>
     <row r="42">
       <c r="B42" s="5" t="inlineStr">
@@ -3922,6 +4111,11 @@
           <t>• Prevenzione: mantenimento su volume alto; Nordic ai livelli massimi del ciclo.</t>
         </is>
       </c>
+      <c r="C42" s="24" t="n"/>
+      <c r="D42" s="24" t="n"/>
+      <c r="E42" s="24" t="n"/>
+      <c r="F42" s="24" t="n"/>
+      <c r="G42" s="25" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -3983,6 +4177,11 @@
           <t>Taper: volume basso, qualità e velocità. Re-test e rifinitura. Obiettivo: massima freschezza e prontezza per la 1ª gara (31/10).</t>
         </is>
       </c>
+      <c r="C5" s="24" t="n"/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="24" t="n"/>
+      <c r="G5" s="25" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
@@ -4626,6 +4825,11 @@
           <t>• Sala: 3×3-5 focus velocità (~80%), niente massimali.</t>
         </is>
       </c>
+      <c r="C38" s="24" t="n"/>
+      <c r="D38" s="24" t="n"/>
+      <c r="E38" s="24" t="n"/>
+      <c r="F38" s="24" t="n"/>
+      <c r="G38" s="25" t="n"/>
     </row>
     <row r="39">
       <c r="B39" s="5" t="inlineStr">
@@ -4633,6 +4837,11 @@
           <t>• Pliometria: solo qualità (CMJ max intent, poche rip.).</t>
         </is>
       </c>
+      <c r="C39" s="24" t="n"/>
+      <c r="D39" s="24" t="n"/>
+      <c r="E39" s="24" t="n"/>
+      <c r="F39" s="24" t="n"/>
+      <c r="G39" s="25" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="5" t="inlineStr">
@@ -4640,6 +4849,11 @@
           <t>• Chiusura con RE-TEST completo (vedi scheda Test &amp; Marker).</t>
         </is>
       </c>
+      <c r="C40" s="24" t="n"/>
+      <c r="D40" s="24" t="n"/>
+      <c r="E40" s="24" t="n"/>
+      <c r="F40" s="24" t="n"/>
+      <c r="G40" s="25" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -5000,6 +5214,9 @@
           <t>• RPE seduta (carico interno) — se sale a pari lavoro esterno = affaticamento.</t>
         </is>
       </c>
+      <c r="C13" s="24" t="n"/>
+      <c r="D13" s="24" t="n"/>
+      <c r="E13" s="25" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="5" t="inlineStr">
@@ -5007,6 +5224,9 @@
           <t>• Wellness breve (sonno, dolori, energia) — soprattutto in un gruppo femminile; autoregolare il carico.</t>
         </is>
       </c>
+      <c r="C14" s="24" t="n"/>
+      <c r="D14" s="24" t="n"/>
+      <c r="E14" s="25" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="5" t="inlineStr">
@@ -5014,6 +5234,9 @@
           <t>• Dolore/fastidio articolare (ginocchio, spalla, caviglia) — STOP e regressione se presente.</t>
         </is>
       </c>
+      <c r="C15" s="24" t="n"/>
+      <c r="D15" s="24" t="n"/>
+      <c r="E15" s="25" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="5" t="inlineStr">
@@ -5021,6 +5244,9 @@
           <t>• Simmetria arti (hop test) — differenza &gt;10-15% = rischio, individualizzare.</t>
         </is>
       </c>
+      <c r="C16" s="24" t="n"/>
+      <c r="D16" s="24" t="n"/>
+      <c r="E16" s="25" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>